<commit_message>
Updated AUS_grids_kan50 model - 2026-09-06 17:49
</commit_message>
<xml_diff>
--- a/VerveStacks_AUS_grids_kan50/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_AUS_grids_kan50/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_AUS_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85A5FB5D-BC8C-4713-9441-704ACA628D1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEAF5432-E54A-484B-97A7-B8345087DE07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25246,7 +25246,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3B7B27E-7915-4268-A5F3-FA6D499E6671}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26BD7420-9C40-48A2-B324-E0FA08FEA904}">
   <dimension ref="B9:H298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -31044,7 +31044,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC9C5050-2CA9-49D5-82BC-72B456BCDB21}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20324267-DE7F-4280-B293-C8A6023387DE}">
   <dimension ref="B9:L298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated AUS_grids_kan50 model - 2026-09-06 18:23
</commit_message>
<xml_diff>
--- a/VerveStacks_AUS_grids_kan50/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_AUS_grids_kan50/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_AUS_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEAF5432-E54A-484B-97A7-B8345087DE07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF3B8DBF-164C-4253-8B73-BE98E70921CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25246,7 +25246,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26BD7420-9C40-48A2-B324-E0FA08FEA904}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDB6814A-9F20-43F0-A466-BECC04F6B0A8}">
   <dimension ref="B9:H298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -31044,7 +31044,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20324267-DE7F-4280-B293-C8A6023387DE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB30B20B-7914-4C97-A287-B5C791587A07}">
   <dimension ref="B9:L298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated AUS_grids_kan50 model - 2026-09-06 23:05
</commit_message>
<xml_diff>
--- a/VerveStacks_AUS_grids_kan50/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_AUS_grids_kan50/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_AUS_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84904E5E-8D71-4260-B018-7EEA3C9EEEB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FB2497A-FD5A-4616-89FA-4AC67144AD4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25273,7 +25273,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A151B40D-8CC4-43EE-9784-0D15FC83369F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{229B6CFB-000B-4016-BDAA-FD6D006B3B8F}">
   <dimension ref="B9:H301"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -31131,7 +31131,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1308E76-9ED3-4C77-92D3-5EC70007784B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD5E4BAC-A827-4954-AE16-EAEA98E38E4B}">
   <dimension ref="B9:L301"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated AUS_grids_kan50 model - 2026-09-07 14:54
</commit_message>
<xml_diff>
--- a/VerveStacks_AUS_grids_kan50/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_AUS_grids_kan50/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_AUS_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99FB901E-FDFA-42FB-B510-2320D2A29034}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E82EFA88-DB7D-4CB1-86E8-D7BEC782BEBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4914,7 +4914,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84EC8663-B1D5-4762-B0AD-569B1CB624A9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D945912A-55D7-4FC4-819A-2266EFA4550B}">
   <dimension ref="B9:L300"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -35690,7 +35690,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B033C26-17E5-4E0B-90CB-E7B07165A0D7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DCF73DF-291D-41CD-B3B0-2EEE7FBACAA8}">
   <dimension ref="B9:H300"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated AUS_grids_kan50 model - 2026-09-07 22:06
</commit_message>
<xml_diff>
--- a/VerveStacks_AUS_grids_kan50/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_AUS_grids_kan50/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_AUS_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E82EFA88-DB7D-4CB1-86E8-D7BEC782BEBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B602E16-EB3A-466B-A428-CB4D6D677EA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4914,7 +4914,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D945912A-55D7-4FC4-819A-2266EFA4550B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26A34495-22B6-4ED4-9CF7-2432AFB5281C}">
   <dimension ref="B9:L300"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -35690,7 +35690,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DCF73DF-291D-41CD-B3B0-2EEE7FBACAA8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77FA3F82-56C8-4FF7-9EAA-A456F757AAFE}">
   <dimension ref="B9:H300"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated AUS_grids_kan50 model - 2026-09-08 00:21
</commit_message>
<xml_diff>
--- a/VerveStacks_AUS_grids_kan50/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_AUS_grids_kan50/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_AUS_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A5B5E66-9D4C-4653-A486-52D438D351F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7958330-FB9C-480C-B804-D328360EDC87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1471,7 +1471,7 @@
     <t>p_PortHedland_AUS</t>
   </si>
   <si>
-    <t>p_AUS42p8S146p2E_AUS</t>
+    <t>p_Hobart_AUS</t>
   </si>
   <si>
     <t>p_Kalgoorlie_AUS</t>
@@ -2377,7 +2377,7 @@
     <t>e_PortHedland_AUS</t>
   </si>
   <si>
-    <t>e_AUS42p8S146p2E_AUS</t>
+    <t>e_Hobart_AUS</t>
   </si>
   <si>
     <t>e_Kalgoorlie_AUS</t>
@@ -3262,7 +3262,7 @@
     <t>AUS-e_PortHedland_AUS</t>
   </si>
   <si>
-    <t>AUS-e_AUS42p8S146p2E_AUS</t>
+    <t>AUS-e_Hobart_AUS</t>
   </si>
   <si>
     <t>AUS-e_Kalgoorlie_AUS</t>
@@ -4932,7 +4932,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A3619EB-FD1B-4C96-9F43-755B5FE548E2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2998290A-40A2-4F49-8504-0379DC41DD2C}">
   <dimension ref="B9:L302"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -35766,7 +35766,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FFE0F01-42FD-47B6-867C-7813486C09DA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE23AFD7-8A34-41C7-8BFB-0386FDFFA2F4}">
   <dimension ref="B9:H302"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -36683,19 +36683,19 @@
         <v>462</v>
       </c>
       <c r="C55">
-        <v>-42.848328268142403</v>
+        <v>-42.823952846681991</v>
       </c>
       <c r="D55">
-        <v>146.17591077698933</v>
+        <v>146.7152693827272</v>
       </c>
       <c r="F55" t="s">
         <v>1059</v>
       </c>
       <c r="G55">
-        <v>-42.848328268142403</v>
+        <v>-42.823952846681991</v>
       </c>
       <c r="H55">
-        <v>146.17591077698933</v>
+        <v>146.7152693827272</v>
       </c>
     </row>
     <row r="56" spans="2:8">
@@ -36783,19 +36783,19 @@
         <v>467</v>
       </c>
       <c r="C60">
-        <v>-41.239472398304343</v>
+        <v>-41.2407776578913</v>
       </c>
       <c r="D60">
-        <v>145.74672600476077</v>
+        <v>145.74657208657698</v>
       </c>
       <c r="F60" t="s">
         <v>1064</v>
       </c>
       <c r="G60">
-        <v>-41.239472398304343</v>
+        <v>-41.2407776578913</v>
       </c>
       <c r="H60">
-        <v>145.74672600476077</v>
+        <v>145.74657208657698</v>
       </c>
     </row>
     <row r="61" spans="2:8">
@@ -37243,19 +37243,19 @@
         <v>490</v>
       </c>
       <c r="C83">
-        <v>-41.86050859336482</v>
+        <v>-41.754650558287658</v>
       </c>
       <c r="D83">
-        <v>147.48956461856997</v>
+        <v>147.51971261676547</v>
       </c>
       <c r="F83" t="s">
         <v>1087</v>
       </c>
       <c r="G83">
-        <v>-41.86050859336482</v>
+        <v>-41.754650558287658</v>
       </c>
       <c r="H83">
-        <v>147.48956461856997</v>
+        <v>147.51971261676547</v>
       </c>
     </row>
     <row r="84" spans="2:8">
@@ -38503,19 +38503,19 @@
         <v>553</v>
       </c>
       <c r="C146">
-        <v>-42.539251485649778</v>
+        <v>-42.677737589053145</v>
       </c>
       <c r="D146">
-        <v>146.61070950534349</v>
+        <v>147.1701068156745</v>
       </c>
       <c r="F146" t="s">
         <v>1150</v>
       </c>
       <c r="G146">
-        <v>-42.539251485649778</v>
+        <v>-42.677737589053145</v>
       </c>
       <c r="H146">
-        <v>146.61070950534349</v>
+        <v>147.1701068156745</v>
       </c>
     </row>
     <row r="147" spans="2:8">
@@ -38723,19 +38723,19 @@
         <v>564</v>
       </c>
       <c r="C157">
-        <v>-41.070134274350721</v>
+        <v>-41.072643681112218</v>
       </c>
       <c r="D157">
-        <v>145.43263864663615</v>
+        <v>145.43305512263535</v>
       </c>
       <c r="F157" t="s">
         <v>1161</v>
       </c>
       <c r="G157">
-        <v>-41.070134274350721</v>
+        <v>-41.072643681112218</v>
       </c>
       <c r="H157">
-        <v>145.43263864663615</v>
+        <v>145.43305512263535</v>
       </c>
     </row>
     <row r="158" spans="2:8">
@@ -39163,19 +39163,19 @@
         <v>586</v>
       </c>
       <c r="C179">
-        <v>-42.094338889464559</v>
+        <v>-41.912687414816389</v>
       </c>
       <c r="D179">
-        <v>147.39311396207361</v>
+        <v>147.4317513167116</v>
       </c>
       <c r="F179" t="s">
         <v>1183</v>
       </c>
       <c r="G179">
-        <v>-42.094338889464559</v>
+        <v>-41.912687414816389</v>
       </c>
       <c r="H179">
-        <v>147.39311396207361</v>
+        <v>147.4317513167116</v>
       </c>
     </row>
     <row r="180" spans="2:8">
@@ -40423,19 +40423,19 @@
         <v>649</v>
       </c>
       <c r="C242">
-        <v>-43.000695831545308</v>
+        <v>-42.735045094737728</v>
       </c>
       <c r="D242">
-        <v>146.97091687570963</v>
+        <v>147.23477366457425</v>
       </c>
       <c r="F242" t="s">
         <v>1246</v>
       </c>
       <c r="G242">
-        <v>-43.000695831545308</v>
+        <v>-42.735045094737728</v>
       </c>
       <c r="H242">
-        <v>146.97091687570963</v>
+        <v>147.23477366457425</v>
       </c>
     </row>
     <row r="243" spans="2:8">
@@ -40643,19 +40643,19 @@
         <v>660</v>
       </c>
       <c r="C253">
-        <v>-40.272839726974297</v>
+        <v>-41.44005143720814</v>
       </c>
       <c r="D253">
-        <v>146.66672296307451</v>
+        <v>144.36113356472447</v>
       </c>
       <c r="F253" t="s">
         <v>1257</v>
       </c>
       <c r="G253">
-        <v>-40.272839726974297</v>
+        <v>-41.44005143720814</v>
       </c>
       <c r="H253">
-        <v>146.66672296307451</v>
+        <v>144.36113356472447</v>
       </c>
     </row>
     <row r="254" spans="2:8">
@@ -40663,19 +40663,19 @@
         <v>661</v>
       </c>
       <c r="C254">
-        <v>-40.546840571798938</v>
+        <v>-40.254914758185407</v>
       </c>
       <c r="D254">
-        <v>144.64697355726699</v>
+        <v>145.97678015008486</v>
       </c>
       <c r="F254" t="s">
         <v>1258</v>
       </c>
       <c r="G254">
-        <v>-40.546840571798938</v>
+        <v>-40.254914758185407</v>
       </c>
       <c r="H254">
-        <v>144.64697355726699</v>
+        <v>145.97678015008486</v>
       </c>
     </row>
     <row r="255" spans="2:8">
@@ -40983,19 +40983,19 @@
         <v>677</v>
       </c>
       <c r="C270">
-        <v>-41.33210911071906</v>
+        <v>-41.089250164550577</v>
       </c>
       <c r="D270">
-        <v>148.55880462471723</v>
+        <v>148.64966281870522</v>
       </c>
       <c r="F270" t="s">
         <v>1274</v>
       </c>
       <c r="G270">
-        <v>-41.33210911071906</v>
+        <v>-41.089250164550577</v>
       </c>
       <c r="H270">
-        <v>148.55880462471723</v>
+        <v>148.64966281870522</v>
       </c>
     </row>
     <row r="271" spans="2:8">
@@ -41583,19 +41583,19 @@
         <v>707</v>
       </c>
       <c r="C300">
-        <v>-43.909028252220295</v>
+        <v>-43.459445564853546</v>
       </c>
       <c r="D300">
-        <v>146.29696618066109</v>
+        <v>147.10370753016318</v>
       </c>
       <c r="F300" t="s">
         <v>1304</v>
       </c>
       <c r="G300">
-        <v>-43.909028252220295</v>
+        <v>-43.459445564853546</v>
       </c>
       <c r="H300">
-        <v>146.29696618066109</v>
+        <v>147.10370753016318</v>
       </c>
     </row>
     <row r="301" spans="2:8">

</xml_diff>

<commit_message>
Updated AUS_grids_kan50 model - 2026-09-08 16:07
</commit_message>
<xml_diff>
--- a/VerveStacks_AUS_grids_kan50/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_AUS_grids_kan50/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_AUS_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7958330-FB9C-480C-B804-D328360EDC87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B9AE1DC-808B-463D-B7CF-FE7844B09502}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1384,6 +1384,9 @@
     <t>p_Tarong_AUS</t>
   </si>
   <si>
+    <t>p_Ipswich_AUS</t>
+  </si>
+  <si>
     <t>p_Bouldercombe_AUS</t>
   </si>
   <si>
@@ -1399,9 +1402,6 @@
     <t>p_Para_AUS</t>
   </si>
   <si>
-    <t>p_Brisbane_AUS</t>
-  </si>
-  <si>
     <t>p_BulliCreek_AUS</t>
   </si>
   <si>
@@ -1468,12 +1468,12 @@
     <t>p_Horsham_AUS</t>
   </si>
   <si>
+    <t>p_Kingston_AUS</t>
+  </si>
+  <si>
     <t>p_PortHedland_AUS</t>
   </si>
   <si>
-    <t>p_Hobart_AUS</t>
-  </si>
-  <si>
     <t>p_Kalgoorlie_AUS</t>
   </si>
   <si>
@@ -2290,6 +2290,9 @@
     <t>e_Tarong_AUS</t>
   </si>
   <si>
+    <t>e_Ipswich_AUS</t>
+  </si>
+  <si>
     <t>e_Bouldercombe_AUS</t>
   </si>
   <si>
@@ -2305,9 +2308,6 @@
     <t>e_Para_AUS</t>
   </si>
   <si>
-    <t>e_Brisbane_AUS</t>
-  </si>
-  <si>
     <t>e_BulliCreek_AUS</t>
   </si>
   <si>
@@ -2374,12 +2374,12 @@
     <t>e_Horsham_AUS</t>
   </si>
   <si>
+    <t>e_Kingston_AUS</t>
+  </si>
+  <si>
     <t>e_PortHedland_AUS</t>
   </si>
   <si>
-    <t>e_Hobart_AUS</t>
-  </si>
-  <si>
     <t>e_Kalgoorlie_AUS</t>
   </si>
   <si>
@@ -3175,6 +3175,9 @@
     <t>AUS-e_Tarong_AUS</t>
   </si>
   <si>
+    <t>AUS-e_Ipswich_AUS</t>
+  </si>
+  <si>
     <t>AUS-e_Bouldercombe_AUS</t>
   </si>
   <si>
@@ -3190,9 +3193,6 @@
     <t>AUS-e_Para_AUS</t>
   </si>
   <si>
-    <t>AUS-e_Brisbane_AUS</t>
-  </si>
-  <si>
     <t>AUS-e_BulliCreek_AUS</t>
   </si>
   <si>
@@ -3259,10 +3259,10 @@
     <t>AUS-e_Horsham_AUS</t>
   </si>
   <si>
+    <t>AUS-e_Kingston_AUS</t>
+  </si>
+  <si>
     <t>AUS-e_PortHedland_AUS</t>
-  </si>
-  <si>
-    <t>AUS-e_Hobart_AUS</t>
   </si>
   <si>
     <t>AUS-e_Kalgoorlie_AUS</t>
@@ -4932,7 +4932,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2998290A-40A2-4F49-8504-0379DC41DD2C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C9EB49D-E06F-478B-85C9-F18994D7B514}">
   <dimension ref="B9:L302"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -5515,7 +5515,7 @@
         <v>710</v>
       </c>
       <c r="H29" t="s">
-        <v>711</v>
+        <v>715</v>
       </c>
       <c r="J29" t="s">
         <v>719</v>
@@ -5544,7 +5544,7 @@
         <v>710</v>
       </c>
       <c r="H30" t="s">
-        <v>716</v>
+        <v>711</v>
       </c>
       <c r="J30" t="s">
         <v>719</v>
@@ -5573,7 +5573,7 @@
         <v>710</v>
       </c>
       <c r="H31" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="J31" t="s">
         <v>719</v>
@@ -6240,7 +6240,7 @@
         <v>710</v>
       </c>
       <c r="H54" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="J54" t="s">
         <v>719</v>
@@ -6269,7 +6269,7 @@
         <v>710</v>
       </c>
       <c r="H55" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="J55" t="s">
         <v>719</v>
@@ -6965,7 +6965,7 @@
         <v>710</v>
       </c>
       <c r="H79" t="s">
-        <v>711</v>
+        <v>715</v>
       </c>
       <c r="J79" t="s">
         <v>719</v>
@@ -6994,7 +6994,7 @@
         <v>710</v>
       </c>
       <c r="H80" t="s">
-        <v>716</v>
+        <v>711</v>
       </c>
       <c r="J80" t="s">
         <v>719</v>
@@ -7023,7 +7023,7 @@
         <v>710</v>
       </c>
       <c r="H81" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="J81" t="s">
         <v>719</v>
@@ -8734,7 +8734,7 @@
         <v>710</v>
       </c>
       <c r="H140" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="J140" t="s">
         <v>719</v>
@@ -8792,7 +8792,7 @@
         <v>710</v>
       </c>
       <c r="H142" t="s">
-        <v>713</v>
+        <v>717</v>
       </c>
       <c r="J142" t="s">
         <v>719</v>
@@ -8908,7 +8908,7 @@
         <v>710</v>
       </c>
       <c r="H146" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="J146" t="s">
         <v>719</v>
@@ -9633,7 +9633,7 @@
         <v>710</v>
       </c>
       <c r="H171" t="s">
-        <v>715</v>
+        <v>711</v>
       </c>
       <c r="J171" t="s">
         <v>719</v>
@@ -9749,7 +9749,7 @@
         <v>710</v>
       </c>
       <c r="H175" t="s">
-        <v>711</v>
+        <v>715</v>
       </c>
       <c r="J175" t="s">
         <v>719</v>
@@ -9778,7 +9778,7 @@
         <v>710</v>
       </c>
       <c r="H176" t="s">
-        <v>716</v>
+        <v>711</v>
       </c>
       <c r="J176" t="s">
         <v>719</v>
@@ -9807,7 +9807,7 @@
         <v>710</v>
       </c>
       <c r="H177" t="s">
-        <v>711</v>
+        <v>716</v>
       </c>
       <c r="J177" t="s">
         <v>719</v>
@@ -11547,7 +11547,7 @@
         <v>710</v>
       </c>
       <c r="H237" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="J237" t="s">
         <v>719</v>
@@ -11634,7 +11634,7 @@
         <v>710</v>
       </c>
       <c r="H240" t="s">
-        <v>717</v>
+        <v>713</v>
       </c>
       <c r="J240" t="s">
         <v>719</v>
@@ -11663,7 +11663,7 @@
         <v>710</v>
       </c>
       <c r="H241" t="s">
-        <v>713</v>
+        <v>717</v>
       </c>
       <c r="J241" t="s">
         <v>719</v>
@@ -11692,7 +11692,7 @@
         <v>710</v>
       </c>
       <c r="H242" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="J242" t="s">
         <v>719</v>
@@ -12156,7 +12156,7 @@
         <v>710</v>
       </c>
       <c r="H258" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="J258" t="s">
         <v>719</v>
@@ -12185,7 +12185,7 @@
         <v>710</v>
       </c>
       <c r="H259" t="s">
-        <v>718</v>
+        <v>716</v>
       </c>
       <c r="J259" t="s">
         <v>719</v>
@@ -35766,7 +35766,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE23AFD7-8A34-41C7-8BFB-0386FDFFA2F4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2ADB422F-9FA9-4998-B303-561D311D6D69}">
   <dimension ref="B9:H302"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -36103,19 +36103,19 @@
         <v>433</v>
       </c>
       <c r="C26">
-        <v>-23.537233256213721</v>
+        <v>-27.541324760522063</v>
       </c>
       <c r="D26">
-        <v>150.48716060704265</v>
+        <v>152.78594479220749</v>
       </c>
       <c r="F26" t="s">
         <v>1030</v>
       </c>
       <c r="G26">
-        <v>-23.537233256213721</v>
+        <v>-27.541324760522063</v>
       </c>
       <c r="H26">
-        <v>150.48716060704265</v>
+        <v>152.78594479220749</v>
       </c>
     </row>
     <row r="27" spans="2:8">
@@ -36123,19 +36123,19 @@
         <v>434</v>
       </c>
       <c r="C27">
-        <v>-24.90133538944163</v>
+        <v>-23.537233256213721</v>
       </c>
       <c r="D27">
-        <v>151.81952564800682</v>
+        <v>150.48716060704265</v>
       </c>
       <c r="F27" t="s">
         <v>1031</v>
       </c>
       <c r="G27">
-        <v>-24.90133538944163</v>
+        <v>-23.537233256213721</v>
       </c>
       <c r="H27">
-        <v>151.81952564800682</v>
+        <v>150.48716060704265</v>
       </c>
     </row>
     <row r="28" spans="2:8">
@@ -36143,19 +36143,19 @@
         <v>435</v>
       </c>
       <c r="C28">
-        <v>-20.499447155592211</v>
+        <v>-24.90133538944163</v>
       </c>
       <c r="D28">
-        <v>147.7754061331616</v>
+        <v>151.81952564800682</v>
       </c>
       <c r="F28" t="s">
         <v>1032</v>
       </c>
       <c r="G28">
-        <v>-20.499447155592211</v>
+        <v>-24.90133538944163</v>
       </c>
       <c r="H28">
-        <v>147.7754061331616</v>
+        <v>151.81952564800682</v>
       </c>
     </row>
     <row r="29" spans="2:8">
@@ -36163,19 +36163,19 @@
         <v>436</v>
       </c>
       <c r="C29">
-        <v>-35.200406760019412</v>
+        <v>-20.499447155592211</v>
       </c>
       <c r="D29">
-        <v>147.39393085110601</v>
+        <v>147.7754061331616</v>
       </c>
       <c r="F29" t="s">
         <v>1033</v>
       </c>
       <c r="G29">
-        <v>-35.200406760019412</v>
+        <v>-20.499447155592211</v>
       </c>
       <c r="H29">
-        <v>147.39393085110601</v>
+        <v>147.7754061331616</v>
       </c>
     </row>
     <row r="30" spans="2:8">
@@ -36183,19 +36183,19 @@
         <v>437</v>
       </c>
       <c r="C30">
-        <v>-34.7354348842319</v>
+        <v>-35.200406760019412</v>
       </c>
       <c r="D30">
-        <v>138.71215621124384</v>
+        <v>147.39393085110601</v>
       </c>
       <c r="F30" t="s">
         <v>1034</v>
       </c>
       <c r="G30">
-        <v>-34.7354348842319</v>
+        <v>-35.200406760019412</v>
       </c>
       <c r="H30">
-        <v>138.71215621124384</v>
+        <v>147.39393085110601</v>
       </c>
     </row>
     <row r="31" spans="2:8">
@@ -36203,19 +36203,19 @@
         <v>438</v>
       </c>
       <c r="C31">
-        <v>-27.732264407857119</v>
+        <v>-34.7354348842319</v>
       </c>
       <c r="D31">
-        <v>152.95633561497641</v>
+        <v>138.71215621124384</v>
       </c>
       <c r="F31" t="s">
         <v>1035</v>
       </c>
       <c r="G31">
-        <v>-27.732264407857119</v>
+        <v>-34.7354348842319</v>
       </c>
       <c r="H31">
-        <v>152.95633561497641</v>
+        <v>138.71215621124384</v>
       </c>
     </row>
     <row r="32" spans="2:8">
@@ -36663,19 +36663,19 @@
         <v>461</v>
       </c>
       <c r="C54">
-        <v>-20.432074971605672</v>
+        <v>-42.829905988893763</v>
       </c>
       <c r="D54">
-        <v>118.54463160000005</v>
+        <v>147.20840569999993</v>
       </c>
       <c r="F54" t="s">
         <v>1058</v>
       </c>
       <c r="G54">
-        <v>-20.432074971605672</v>
+        <v>-42.829905988893763</v>
       </c>
       <c r="H54">
-        <v>118.54463160000005</v>
+        <v>147.20840569999993</v>
       </c>
     </row>
     <row r="55" spans="2:8">
@@ -36683,19 +36683,19 @@
         <v>462</v>
       </c>
       <c r="C55">
-        <v>-42.823952846681991</v>
+        <v>-20.432074971605672</v>
       </c>
       <c r="D55">
-        <v>146.7152693827272</v>
+        <v>118.54463160000005</v>
       </c>
       <c r="F55" t="s">
         <v>1059</v>
       </c>
       <c r="G55">
-        <v>-42.823952846681991</v>
+        <v>-20.432074971605672</v>
       </c>
       <c r="H55">
-        <v>146.7152693827272</v>
+        <v>118.54463160000005</v>
       </c>
     </row>
     <row r="56" spans="2:8">
@@ -36863,19 +36863,19 @@
         <v>471</v>
       </c>
       <c r="C64">
-        <v>-30.507071736111641</v>
+        <v>-30.506116756678612</v>
       </c>
       <c r="D64">
-        <v>150.70172534099848</v>
+        <v>150.70502233548291</v>
       </c>
       <c r="F64" t="s">
         <v>1068</v>
       </c>
       <c r="G64">
-        <v>-30.507071736111641</v>
+        <v>-30.506116756678612</v>
       </c>
       <c r="H64">
-        <v>150.70172534099848</v>
+        <v>150.70502233548291</v>
       </c>
     </row>
     <row r="65" spans="2:8">
@@ -37063,19 +37063,19 @@
         <v>481</v>
       </c>
       <c r="C74">
-        <v>-23.706875486581438</v>
+        <v>-28.24304589666794</v>
       </c>
       <c r="D74">
-        <v>150.15732905181272</v>
+        <v>152.80647923996878</v>
       </c>
       <c r="F74" t="s">
         <v>1078</v>
       </c>
       <c r="G74">
-        <v>-23.706875486581438</v>
+        <v>-28.24304589666794</v>
       </c>
       <c r="H74">
-        <v>150.15732905181272</v>
+        <v>152.80647923996878</v>
       </c>
     </row>
     <row r="75" spans="2:8">
@@ -37083,19 +37083,19 @@
         <v>482</v>
       </c>
       <c r="C75">
-        <v>-25.411178903352639</v>
+        <v>-23.706875486581438</v>
       </c>
       <c r="D75">
-        <v>151.4718066142166</v>
+        <v>150.15732905181272</v>
       </c>
       <c r="F75" t="s">
         <v>1079</v>
       </c>
       <c r="G75">
-        <v>-25.411178903352639</v>
+        <v>-23.706875486581438</v>
       </c>
       <c r="H75">
-        <v>151.4718066142166</v>
+        <v>150.15732905181272</v>
       </c>
     </row>
     <row r="76" spans="2:8">
@@ -37103,19 +37103,19 @@
         <v>483</v>
       </c>
       <c r="C76">
-        <v>-20.994143017659859</v>
+        <v>-25.411178903352639</v>
       </c>
       <c r="D76">
-        <v>146.43171849829355</v>
+        <v>151.4718066142166</v>
       </c>
       <c r="F76" t="s">
         <v>1080</v>
       </c>
       <c r="G76">
-        <v>-20.994143017659859</v>
+        <v>-25.411178903352639</v>
       </c>
       <c r="H76">
-        <v>146.43171849829355</v>
+        <v>151.4718066142166</v>
       </c>
     </row>
     <row r="77" spans="2:8">
@@ -37123,19 +37123,19 @@
         <v>484</v>
       </c>
       <c r="C77">
-        <v>-23.911108657321289</v>
+        <v>-20.994143017659859</v>
       </c>
       <c r="D77">
-        <v>143.01659064084205</v>
+        <v>146.43171849829355</v>
       </c>
       <c r="F77" t="s">
         <v>1081</v>
       </c>
       <c r="G77">
-        <v>-23.911108657321289</v>
+        <v>-20.994143017659859</v>
       </c>
       <c r="H77">
-        <v>143.01659064084205</v>
+        <v>146.43171849829355</v>
       </c>
     </row>
     <row r="78" spans="2:8">
@@ -37143,19 +37143,19 @@
         <v>485</v>
       </c>
       <c r="C78">
-        <v>-22.380981243555336</v>
+        <v>-23.911108657321289</v>
       </c>
       <c r="D78">
-        <v>144.14104615068234</v>
+        <v>143.01659064084205</v>
       </c>
       <c r="F78" t="s">
         <v>1082</v>
       </c>
       <c r="G78">
-        <v>-22.380981243555336</v>
+        <v>-23.911108657321289</v>
       </c>
       <c r="H78">
-        <v>144.14104615068234</v>
+        <v>143.01659064084205</v>
       </c>
     </row>
     <row r="79" spans="2:8">
@@ -37163,19 +37163,19 @@
         <v>486</v>
       </c>
       <c r="C79">
-        <v>-35.953929114813228</v>
+        <v>-22.380981243555336</v>
       </c>
       <c r="D79">
-        <v>146.94281184898847</v>
+        <v>144.14104615068234</v>
       </c>
       <c r="F79" t="s">
         <v>1083</v>
       </c>
       <c r="G79">
-        <v>-35.953929114813228</v>
+        <v>-22.380981243555336</v>
       </c>
       <c r="H79">
-        <v>146.94281184898847</v>
+        <v>144.14104615068234</v>
       </c>
     </row>
     <row r="80" spans="2:8">
@@ -37183,19 +37183,19 @@
         <v>487</v>
       </c>
       <c r="C80">
-        <v>-35.731086944716644</v>
+        <v>-35.953929114813228</v>
       </c>
       <c r="D80">
-        <v>139.31840264795321</v>
+        <v>146.94281184898847</v>
       </c>
       <c r="F80" t="s">
         <v>1084</v>
       </c>
       <c r="G80">
-        <v>-35.731086944716644</v>
+        <v>-35.953929114813228</v>
       </c>
       <c r="H80">
-        <v>139.31840264795321</v>
+        <v>146.94281184898847</v>
       </c>
     </row>
     <row r="81" spans="2:8">
@@ -37203,19 +37203,19 @@
         <v>488</v>
       </c>
       <c r="C81">
-        <v>-28.248182600001183</v>
+        <v>-35.731086944716644</v>
       </c>
       <c r="D81">
-        <v>152.8095039798896</v>
+        <v>139.31840264795321</v>
       </c>
       <c r="F81" t="s">
         <v>1085</v>
       </c>
       <c r="G81">
-        <v>-28.248182600001183</v>
+        <v>-35.731086944716644</v>
       </c>
       <c r="H81">
-        <v>152.8095039798896</v>
+        <v>139.31840264795321</v>
       </c>
     </row>
     <row r="82" spans="2:8">
@@ -37243,19 +37243,19 @@
         <v>490</v>
       </c>
       <c r="C83">
-        <v>-41.754650558287658</v>
+        <v>-41.740655806615202</v>
       </c>
       <c r="D83">
-        <v>147.51971261676547</v>
+        <v>147.48606991865145</v>
       </c>
       <c r="F83" t="s">
         <v>1087</v>
       </c>
       <c r="G83">
-        <v>-41.754650558287658</v>
+        <v>-41.740655806615202</v>
       </c>
       <c r="H83">
-        <v>147.51971261676547</v>
+        <v>147.48606991865145</v>
       </c>
     </row>
     <row r="84" spans="2:8">
@@ -38383,19 +38383,19 @@
         <v>547</v>
       </c>
       <c r="C140">
-        <v>-19.148753079902079</v>
+        <v>-42.609106537819358</v>
       </c>
       <c r="D140">
-        <v>130.44549037437517</v>
+        <v>147.41425715594278</v>
       </c>
       <c r="F140" t="s">
         <v>1144</v>
       </c>
       <c r="G140">
-        <v>-19.148753079902079</v>
+        <v>-42.609106537819358</v>
       </c>
       <c r="H140">
-        <v>130.44549037437517</v>
+        <v>147.41425715594278</v>
       </c>
     </row>
     <row r="141" spans="2:8">
@@ -38403,19 +38403,19 @@
         <v>548</v>
       </c>
       <c r="C141">
-        <v>-15.336686243625843</v>
+        <v>-19.148753079902079</v>
       </c>
       <c r="D141">
-        <v>130.21666041483596</v>
+        <v>130.44549037437517</v>
       </c>
       <c r="F141" t="s">
         <v>1145</v>
       </c>
       <c r="G141">
-        <v>-15.336686243625843</v>
+        <v>-19.148753079902079</v>
       </c>
       <c r="H141">
-        <v>130.21666041483596</v>
+        <v>130.44549037437517</v>
       </c>
     </row>
     <row r="142" spans="2:8">
@@ -38423,19 +38423,19 @@
         <v>549</v>
       </c>
       <c r="C142">
-        <v>-20.825706306232721</v>
+        <v>-15.336686243625843</v>
       </c>
       <c r="D142">
-        <v>119.58806566385246</v>
+        <v>130.21666041483596</v>
       </c>
       <c r="F142" t="s">
         <v>1146</v>
       </c>
       <c r="G142">
-        <v>-20.825706306232721</v>
+        <v>-15.336686243625843</v>
       </c>
       <c r="H142">
-        <v>119.58806566385246</v>
+        <v>130.21666041483596</v>
       </c>
     </row>
     <row r="143" spans="2:8">
@@ -38443,19 +38443,19 @@
         <v>550</v>
       </c>
       <c r="C143">
-        <v>-19.907342783485745</v>
+        <v>-20.825706306232721</v>
       </c>
       <c r="D143">
-        <v>123.07722410756404</v>
+        <v>119.58806566385246</v>
       </c>
       <c r="F143" t="s">
         <v>1147</v>
       </c>
       <c r="G143">
-        <v>-19.907342783485745</v>
+        <v>-20.825706306232721</v>
       </c>
       <c r="H143">
-        <v>123.07722410756404</v>
+        <v>119.58806566385246</v>
       </c>
     </row>
     <row r="144" spans="2:8">
@@ -38463,19 +38463,19 @@
         <v>551</v>
       </c>
       <c r="C144">
-        <v>-16.778364179633666</v>
+        <v>-19.907342783485745</v>
       </c>
       <c r="D144">
-        <v>126.86620324681024</v>
+        <v>123.07722410756404</v>
       </c>
       <c r="F144" t="s">
         <v>1148</v>
       </c>
       <c r="G144">
-        <v>-16.778364179633666</v>
+        <v>-19.907342783485745</v>
       </c>
       <c r="H144">
-        <v>126.86620324681024</v>
+        <v>123.07722410756404</v>
       </c>
     </row>
     <row r="145" spans="2:8">
@@ -38483,19 +38483,19 @@
         <v>552</v>
       </c>
       <c r="C145">
-        <v>-19.57556420488984</v>
+        <v>-16.778364179633666</v>
       </c>
       <c r="D145">
-        <v>126.68911386447304</v>
+        <v>126.86620324681024</v>
       </c>
       <c r="F145" t="s">
         <v>1149</v>
       </c>
       <c r="G145">
-        <v>-19.57556420488984</v>
+        <v>-16.778364179633666</v>
       </c>
       <c r="H145">
-        <v>126.68911386447304</v>
+        <v>126.86620324681024</v>
       </c>
     </row>
     <row r="146" spans="2:8">
@@ -38503,19 +38503,19 @@
         <v>553</v>
       </c>
       <c r="C146">
-        <v>-42.677737589053145</v>
+        <v>-19.57556420488984</v>
       </c>
       <c r="D146">
-        <v>147.1701068156745</v>
+        <v>126.68911386447304</v>
       </c>
       <c r="F146" t="s">
         <v>1150</v>
       </c>
       <c r="G146">
-        <v>-42.677737589053145</v>
+        <v>-19.57556420488984</v>
       </c>
       <c r="H146">
-        <v>147.1701068156745</v>
+        <v>126.68911386447304</v>
       </c>
     </row>
     <row r="147" spans="2:8">
@@ -38803,19 +38803,19 @@
         <v>568</v>
       </c>
       <c r="C161">
-        <v>-30.52001579209675</v>
+        <v>-30.518528831413143</v>
       </c>
       <c r="D161">
-        <v>150.9301046692855</v>
+        <v>150.93476814193207</v>
       </c>
       <c r="F161" t="s">
         <v>1165</v>
       </c>
       <c r="G161">
-        <v>-30.52001579209675</v>
+        <v>-30.518528831413143</v>
       </c>
       <c r="H161">
-        <v>150.9301046692855</v>
+        <v>150.93476814193207</v>
       </c>
     </row>
     <row r="162" spans="2:8">
@@ -39003,19 +39003,19 @@
         <v>578</v>
       </c>
       <c r="C171">
-        <v>-23.693112920968051</v>
+        <v>-28.276244191915151</v>
       </c>
       <c r="D171">
-        <v>150.24713680163202</v>
+        <v>152.51317424828557</v>
       </c>
       <c r="F171" t="s">
         <v>1175</v>
       </c>
       <c r="G171">
-        <v>-23.693112920968051</v>
+        <v>-28.276244191915151</v>
       </c>
       <c r="H171">
-        <v>150.24713680163202</v>
+        <v>152.51317424828557</v>
       </c>
     </row>
     <row r="172" spans="2:8">
@@ -39023,19 +39023,19 @@
         <v>579</v>
       </c>
       <c r="C172">
-        <v>-25.37400675796134</v>
+        <v>-23.693112920968051</v>
       </c>
       <c r="D172">
-        <v>151.61716576352794</v>
+        <v>150.24713680163202</v>
       </c>
       <c r="F172" t="s">
         <v>1176</v>
       </c>
       <c r="G172">
-        <v>-25.37400675796134</v>
+        <v>-23.693112920968051</v>
       </c>
       <c r="H172">
-        <v>151.61716576352794</v>
+        <v>150.24713680163202</v>
       </c>
     </row>
     <row r="173" spans="2:8">
@@ -39043,19 +39043,19 @@
         <v>580</v>
       </c>
       <c r="C173">
-        <v>-23.419388107531574</v>
+        <v>-25.37400675796134</v>
       </c>
       <c r="D173">
-        <v>143.35412326528009</v>
+        <v>151.61716576352794</v>
       </c>
       <c r="F173" t="s">
         <v>1177</v>
       </c>
       <c r="G173">
-        <v>-23.419388107531574</v>
+        <v>-25.37400675796134</v>
       </c>
       <c r="H173">
-        <v>143.35412326528009</v>
+        <v>151.61716576352794</v>
       </c>
     </row>
     <row r="174" spans="2:8">
@@ -39063,19 +39063,19 @@
         <v>581</v>
       </c>
       <c r="C174">
-        <v>-21.882733173886301</v>
+        <v>-23.419388107531574</v>
       </c>
       <c r="D174">
-        <v>144.78502894446973</v>
+        <v>143.35412326528009</v>
       </c>
       <c r="F174" t="s">
         <v>1178</v>
       </c>
       <c r="G174">
-        <v>-21.882733173886301</v>
+        <v>-23.419388107531574</v>
       </c>
       <c r="H174">
-        <v>144.78502894446973</v>
+        <v>143.35412326528009</v>
       </c>
     </row>
     <row r="175" spans="2:8">
@@ -39083,19 +39083,19 @@
         <v>582</v>
       </c>
       <c r="C175">
-        <v>-35.479752937238217</v>
+        <v>-21.882733173886301</v>
       </c>
       <c r="D175">
-        <v>147.21725198745645</v>
+        <v>144.78502894446973</v>
       </c>
       <c r="F175" t="s">
         <v>1179</v>
       </c>
       <c r="G175">
-        <v>-35.479752937238217</v>
+        <v>-21.882733173886301</v>
       </c>
       <c r="H175">
-        <v>147.21725198745645</v>
+        <v>144.78502894446973</v>
       </c>
     </row>
     <row r="176" spans="2:8">
@@ -39103,19 +39103,19 @@
         <v>583</v>
       </c>
       <c r="C176">
-        <v>-35.629567001716929</v>
+        <v>-35.479752937238217</v>
       </c>
       <c r="D176">
-        <v>139.19580294835177</v>
+        <v>147.21725198745645</v>
       </c>
       <c r="F176" t="s">
         <v>1180</v>
       </c>
       <c r="G176">
-        <v>-35.629567001716929</v>
+        <v>-35.479752937238217</v>
       </c>
       <c r="H176">
-        <v>139.19580294835177</v>
+        <v>147.21725198745645</v>
       </c>
     </row>
     <row r="177" spans="2:8">
@@ -39123,19 +39123,19 @@
         <v>584</v>
       </c>
       <c r="C177">
-        <v>-28.289668493542941</v>
+        <v>-35.629567001716929</v>
       </c>
       <c r="D177">
-        <v>152.52412221723841</v>
+        <v>139.19580294835177</v>
       </c>
       <c r="F177" t="s">
         <v>1181</v>
       </c>
       <c r="G177">
-        <v>-28.289668493542941</v>
+        <v>-35.629567001716929</v>
       </c>
       <c r="H177">
-        <v>152.52412221723841</v>
+        <v>139.19580294835177</v>
       </c>
     </row>
     <row r="178" spans="2:8">
@@ -39163,19 +39163,19 @@
         <v>586</v>
       </c>
       <c r="C179">
-        <v>-41.912687414816389</v>
+        <v>-41.896128682730868</v>
       </c>
       <c r="D179">
-        <v>147.4317513167116</v>
+        <v>147.40204885581329</v>
       </c>
       <c r="F179" t="s">
         <v>1183</v>
       </c>
       <c r="G179">
-        <v>-41.912687414816389</v>
+        <v>-41.896128682730868</v>
       </c>
       <c r="H179">
-        <v>147.4317513167116</v>
+        <v>147.40204885581329</v>
       </c>
     </row>
     <row r="180" spans="2:8">
@@ -40323,19 +40323,19 @@
         <v>644</v>
       </c>
       <c r="C237">
-        <v>-18.602592489260651</v>
+        <v>-42.675172685233107</v>
       </c>
       <c r="D237">
-        <v>123.0900307495962</v>
+        <v>147.33244449422352</v>
       </c>
       <c r="F237" t="s">
         <v>1241</v>
       </c>
       <c r="G237">
-        <v>-18.602592489260651</v>
+        <v>-42.675172685233107</v>
       </c>
       <c r="H237">
-        <v>123.0900307495962</v>
+        <v>147.33244449422352</v>
       </c>
     </row>
     <row r="238" spans="2:8">
@@ -40343,19 +40343,19 @@
         <v>645</v>
       </c>
       <c r="C238">
-        <v>-20.355566838375449</v>
+        <v>-18.602592489260651</v>
       </c>
       <c r="D238">
-        <v>122.54308312197736</v>
+        <v>123.0900307495962</v>
       </c>
       <c r="F238" t="s">
         <v>1242</v>
       </c>
       <c r="G238">
-        <v>-20.355566838375449</v>
+        <v>-18.602592489260651</v>
       </c>
       <c r="H238">
-        <v>122.54308312197736</v>
+        <v>123.0900307495962</v>
       </c>
     </row>
     <row r="239" spans="2:8">
@@ -40363,19 +40363,19 @@
         <v>646</v>
       </c>
       <c r="C239">
-        <v>-19.496163382311977</v>
+        <v>-20.355566838375449</v>
       </c>
       <c r="D239">
-        <v>128.22766529346336</v>
+        <v>122.54308312197736</v>
       </c>
       <c r="F239" t="s">
         <v>1243</v>
       </c>
       <c r="G239">
-        <v>-19.496163382311977</v>
+        <v>-20.355566838375449</v>
       </c>
       <c r="H239">
-        <v>128.22766529346336</v>
+        <v>122.54308312197736</v>
       </c>
     </row>
     <row r="240" spans="2:8">
@@ -40383,19 +40383,19 @@
         <v>647</v>
       </c>
       <c r="C240">
-        <v>-14.565317050693372</v>
+        <v>-19.496163382311977</v>
       </c>
       <c r="D240">
-        <v>129.86196084560535</v>
+        <v>128.22766529346336</v>
       </c>
       <c r="F240" t="s">
         <v>1244</v>
       </c>
       <c r="G240">
-        <v>-14.565317050693372</v>
+        <v>-19.496163382311977</v>
       </c>
       <c r="H240">
-        <v>129.86196084560535</v>
+        <v>128.22766529346336</v>
       </c>
     </row>
     <row r="241" spans="2:8">
@@ -40403,19 +40403,19 @@
         <v>648</v>
       </c>
       <c r="C241">
-        <v>-17.866548200273396</v>
+        <v>-14.565317050693372</v>
       </c>
       <c r="D241">
-        <v>126.43376235886116</v>
+        <v>129.86196084560535</v>
       </c>
       <c r="F241" t="s">
         <v>1245</v>
       </c>
       <c r="G241">
-        <v>-17.866548200273396</v>
+        <v>-14.565317050693372</v>
       </c>
       <c r="H241">
-        <v>126.43376235886116</v>
+        <v>129.86196084560535</v>
       </c>
     </row>
     <row r="242" spans="2:8">
@@ -40423,19 +40423,19 @@
         <v>649</v>
       </c>
       <c r="C242">
-        <v>-42.735045094737728</v>
+        <v>-17.866548200273396</v>
       </c>
       <c r="D242">
-        <v>147.23477366457425</v>
+        <v>126.43376235886116</v>
       </c>
       <c r="F242" t="s">
         <v>1246</v>
       </c>
       <c r="G242">
-        <v>-42.735045094737728</v>
+        <v>-17.866548200273396</v>
       </c>
       <c r="H242">
-        <v>147.23477366457425</v>
+        <v>126.43376235886116</v>
       </c>
     </row>
     <row r="243" spans="2:8">
@@ -40623,19 +40623,19 @@
         <v>659</v>
       </c>
       <c r="C252">
-        <v>-34.917150029871202</v>
+        <v>-35.070026612914461</v>
       </c>
       <c r="D252">
-        <v>116.44753624908248</v>
+        <v>118.5085945386015</v>
       </c>
       <c r="F252" t="s">
         <v>1256</v>
       </c>
       <c r="G252">
-        <v>-34.917150029871202</v>
+        <v>-35.070026612914461</v>
       </c>
       <c r="H252">
-        <v>116.44753624908248</v>
+        <v>118.5085945386015</v>
       </c>
     </row>
     <row r="253" spans="2:8">
@@ -40643,19 +40643,19 @@
         <v>660</v>
       </c>
       <c r="C253">
-        <v>-41.44005143720814</v>
+        <v>-34.743596006842388</v>
       </c>
       <c r="D253">
-        <v>144.36113356472447</v>
+        <v>115.45951859019976</v>
       </c>
       <c r="F253" t="s">
         <v>1257</v>
       </c>
       <c r="G253">
-        <v>-41.44005143720814</v>
+        <v>-34.743596006842388</v>
       </c>
       <c r="H253">
-        <v>144.36113356472447</v>
+        <v>115.45951859019976</v>
       </c>
     </row>
     <row r="254" spans="2:8">
@@ -40663,19 +40663,19 @@
         <v>661</v>
       </c>
       <c r="C254">
-        <v>-40.254914758185407</v>
+        <v>-40.224745480761946</v>
       </c>
       <c r="D254">
-        <v>145.97678015008486</v>
+        <v>146.38887677493818</v>
       </c>
       <c r="F254" t="s">
         <v>1258</v>
       </c>
       <c r="G254">
-        <v>-40.254914758185407</v>
+        <v>-40.224745480761946</v>
       </c>
       <c r="H254">
-        <v>145.97678015008486</v>
+        <v>146.38887677493818</v>
       </c>
     </row>
     <row r="255" spans="2:8">
@@ -40683,19 +40683,19 @@
         <v>662</v>
       </c>
       <c r="C255">
-        <v>-39.257876116339148</v>
+        <v>-41.062297982110003</v>
       </c>
       <c r="D255">
-        <v>143.87674213215473</v>
+        <v>144.35963098272583</v>
       </c>
       <c r="F255" t="s">
         <v>1259</v>
       </c>
       <c r="G255">
-        <v>-39.257876116339148</v>
+        <v>-41.062297982110003</v>
       </c>
       <c r="H255">
-        <v>143.87674213215473</v>
+        <v>144.35963098272583</v>
       </c>
     </row>
     <row r="256" spans="2:8">
@@ -40703,19 +40703,19 @@
         <v>663</v>
       </c>
       <c r="C256">
-        <v>-21.252254703658771</v>
+        <v>-39.257876116339148</v>
       </c>
       <c r="D256">
-        <v>150.90399697993092</v>
+        <v>143.87674213215473</v>
       </c>
       <c r="F256" t="s">
         <v>1260</v>
       </c>
       <c r="G256">
-        <v>-21.252254703658771</v>
+        <v>-39.257876116339148</v>
       </c>
       <c r="H256">
-        <v>150.90399697993092</v>
+        <v>143.87674213215473</v>
       </c>
     </row>
     <row r="257" spans="2:8">
@@ -40723,19 +40723,19 @@
         <v>664</v>
       </c>
       <c r="C257">
-        <v>-30.859626845395809</v>
+        <v>-21.252254703658771</v>
       </c>
       <c r="D257">
-        <v>153.37306950018458</v>
+        <v>150.90399697993092</v>
       </c>
       <c r="F257" t="s">
         <v>1261</v>
       </c>
       <c r="G257">
-        <v>-30.859626845395809</v>
+        <v>-21.252254703658771</v>
       </c>
       <c r="H257">
-        <v>153.37306950018458</v>
+        <v>150.90399697993092</v>
       </c>
     </row>
     <row r="258" spans="2:8">
@@ -40743,19 +40743,19 @@
         <v>665</v>
       </c>
       <c r="C258">
-        <v>-32.743780387632853</v>
+        <v>-30.56757638507419</v>
       </c>
       <c r="D258">
-        <v>137.75207579058173</v>
+        <v>153.6896898968202</v>
       </c>
       <c r="F258" t="s">
         <v>1262</v>
       </c>
       <c r="G258">
-        <v>-32.743780387632853</v>
+        <v>-30.56757638507419</v>
       </c>
       <c r="H258">
-        <v>137.75207579058173</v>
+        <v>153.6896898968202</v>
       </c>
     </row>
     <row r="259" spans="2:8">
@@ -40763,19 +40763,19 @@
         <v>666</v>
       </c>
       <c r="C259">
-        <v>-34.227843031724603</v>
+        <v>-32.743780387632853</v>
       </c>
       <c r="D259">
-        <v>133.82287060397272</v>
+        <v>137.75207579058173</v>
       </c>
       <c r="F259" t="s">
         <v>1263</v>
       </c>
       <c r="G259">
-        <v>-34.227843031724603</v>
+        <v>-32.743780387632853</v>
       </c>
       <c r="H259">
-        <v>133.82287060397272</v>
+        <v>137.75207579058173</v>
       </c>
     </row>
     <row r="260" spans="2:8">
@@ -40783,19 +40783,19 @@
         <v>667</v>
       </c>
       <c r="C260">
-        <v>-21.199688649197544</v>
+        <v>-34.227843031724603</v>
       </c>
       <c r="D260">
-        <v>150.32141234786266</v>
+        <v>133.82287060397272</v>
       </c>
       <c r="F260" t="s">
         <v>1264</v>
       </c>
       <c r="G260">
-        <v>-21.199688649197544</v>
+        <v>-34.227843031724603</v>
       </c>
       <c r="H260">
-        <v>150.32141234786266</v>
+        <v>133.82287060397272</v>
       </c>
     </row>
     <row r="261" spans="2:8">
@@ -40803,19 +40803,19 @@
         <v>668</v>
       </c>
       <c r="C261">
-        <v>-19.943795597851125</v>
+        <v>-21.199688649197544</v>
       </c>
       <c r="D261">
-        <v>150.81900140649941</v>
+        <v>150.32141234786266</v>
       </c>
       <c r="F261" t="s">
         <v>1265</v>
       </c>
       <c r="G261">
-        <v>-19.943795597851125</v>
+        <v>-21.199688649197544</v>
       </c>
       <c r="H261">
-        <v>150.81900140649941</v>
+        <v>150.32141234786266</v>
       </c>
     </row>
     <row r="262" spans="2:8">
@@ -40823,19 +40823,19 @@
         <v>669</v>
       </c>
       <c r="C262">
-        <v>-25.92492989840304</v>
+        <v>-19.943795597851125</v>
       </c>
       <c r="D262">
-        <v>153.55763832618015</v>
+        <v>150.81900140649941</v>
       </c>
       <c r="F262" t="s">
         <v>1266</v>
       </c>
       <c r="G262">
-        <v>-25.92492989840304</v>
+        <v>-19.943795597851125</v>
       </c>
       <c r="H262">
-        <v>153.55763832618015</v>
+        <v>150.81900140649941</v>
       </c>
     </row>
     <row r="263" spans="2:8">
@@ -40843,19 +40843,19 @@
         <v>670</v>
       </c>
       <c r="C263">
-        <v>-21.50731377536102</v>
+        <v>-27.062670728927419</v>
       </c>
       <c r="D263">
-        <v>151.46867878644642</v>
+        <v>153.65346669501773</v>
       </c>
       <c r="F263" t="s">
         <v>1267</v>
       </c>
       <c r="G263">
-        <v>-21.50731377536102</v>
+        <v>-27.062670728927419</v>
       </c>
       <c r="H263">
-        <v>151.46867878644642</v>
+        <v>153.65346669501773</v>
       </c>
     </row>
     <row r="264" spans="2:8">
@@ -40863,19 +40863,19 @@
         <v>671</v>
       </c>
       <c r="C264">
-        <v>-23.608887736048747</v>
+        <v>-21.50731377536102</v>
       </c>
       <c r="D264">
-        <v>153.73370306869481</v>
+        <v>151.46867878644642</v>
       </c>
       <c r="F264" t="s">
         <v>1268</v>
       </c>
       <c r="G264">
-        <v>-23.608887736048747</v>
+        <v>-21.50731377536102</v>
       </c>
       <c r="H264">
-        <v>153.73370306869481</v>
+        <v>151.46867878644642</v>
       </c>
     </row>
     <row r="265" spans="2:8">
@@ -40883,19 +40883,19 @@
         <v>672</v>
       </c>
       <c r="C265">
-        <v>-17.040567652389406</v>
+        <v>-23.608887736048747</v>
       </c>
       <c r="D265">
-        <v>150.57744483884846</v>
+        <v>153.73370306869481</v>
       </c>
       <c r="F265" t="s">
         <v>1269</v>
       </c>
       <c r="G265">
-        <v>-17.040567652389406</v>
+        <v>-23.608887736048747</v>
       </c>
       <c r="H265">
-        <v>150.57744483884846</v>
+        <v>153.73370306869481</v>
       </c>
     </row>
     <row r="266" spans="2:8">
@@ -40903,19 +40903,19 @@
         <v>673</v>
       </c>
       <c r="C266">
-        <v>-18.721877322770485</v>
+        <v>-17.040567652389406</v>
       </c>
       <c r="D266">
-        <v>149.21297177481156</v>
+        <v>150.57744483884846</v>
       </c>
       <c r="F266" t="s">
         <v>1270</v>
       </c>
       <c r="G266">
-        <v>-18.721877322770485</v>
+        <v>-17.040567652389406</v>
       </c>
       <c r="H266">
-        <v>149.21297177481156</v>
+        <v>150.57744483884846</v>
       </c>
     </row>
     <row r="267" spans="2:8">
@@ -40923,19 +40923,19 @@
         <v>674</v>
       </c>
       <c r="C267">
-        <v>-35.521402273625938</v>
+        <v>-18.721877322770485</v>
       </c>
       <c r="D267">
-        <v>135.81882012006892</v>
+        <v>149.21297177481156</v>
       </c>
       <c r="F267" t="s">
         <v>1271</v>
       </c>
       <c r="G267">
-        <v>-35.521402273625938</v>
+        <v>-18.721877322770485</v>
       </c>
       <c r="H267">
-        <v>135.81882012006892</v>
+        <v>149.21297177481156</v>
       </c>
     </row>
     <row r="268" spans="2:8">
@@ -40943,19 +40943,19 @@
         <v>675</v>
       </c>
       <c r="C268">
-        <v>-36.635585635401441</v>
+        <v>-35.521402273625938</v>
       </c>
       <c r="D268">
-        <v>138.0138906141494</v>
+        <v>135.81882012006892</v>
       </c>
       <c r="F268" t="s">
         <v>1272</v>
       </c>
       <c r="G268">
-        <v>-36.635585635401441</v>
+        <v>-35.521402273625938</v>
       </c>
       <c r="H268">
-        <v>138.0138906141494</v>
+        <v>135.81882012006892</v>
       </c>
     </row>
     <row r="269" spans="2:8">
@@ -40963,19 +40963,19 @@
         <v>676</v>
       </c>
       <c r="C269">
-        <v>-27.74890644111397</v>
+        <v>-36.635585635401441</v>
       </c>
       <c r="D269">
-        <v>153.78400128986024</v>
+        <v>138.0138906141494</v>
       </c>
       <c r="F269" t="s">
         <v>1273</v>
       </c>
       <c r="G269">
-        <v>-27.74890644111397</v>
+        <v>-36.635585635401441</v>
       </c>
       <c r="H269">
-        <v>153.78400128986024</v>
+        <v>138.0138906141494</v>
       </c>
     </row>
     <row r="270" spans="2:8">
@@ -40983,19 +40983,19 @@
         <v>677</v>
       </c>
       <c r="C270">
-        <v>-41.089250164550577</v>
+        <v>-40.739731140552188</v>
       </c>
       <c r="D270">
-        <v>148.64966281870522</v>
+        <v>148.68640459473278</v>
       </c>
       <c r="F270" t="s">
         <v>1274</v>
       </c>
       <c r="G270">
-        <v>-41.089250164550577</v>
+        <v>-40.739731140552188</v>
       </c>
       <c r="H270">
-        <v>148.64966281870522</v>
+        <v>148.68640459473278</v>
       </c>
     </row>
     <row r="271" spans="2:8">
@@ -41523,19 +41523,19 @@
         <v>704</v>
       </c>
       <c r="C297">
-        <v>-17.977932221868844</v>
+        <v>-43.476483100222218</v>
       </c>
       <c r="D297">
-        <v>119.67814798329256</v>
+        <v>147.06278669756466</v>
       </c>
       <c r="F297" t="s">
         <v>1301</v>
       </c>
       <c r="G297">
-        <v>-17.977932221868844</v>
+        <v>-43.476483100222218</v>
       </c>
       <c r="H297">
-        <v>119.67814798329256</v>
+        <v>147.06278669756466</v>
       </c>
     </row>
     <row r="298" spans="2:8">
@@ -41543,19 +41543,19 @@
         <v>705</v>
       </c>
       <c r="C298">
-        <v>-10.13254267953079</v>
+        <v>-17.977932221868844</v>
       </c>
       <c r="D298">
-        <v>130.24318545304698</v>
+        <v>119.67814798329256</v>
       </c>
       <c r="F298" t="s">
         <v>1302</v>
       </c>
       <c r="G298">
-        <v>-10.13254267953079</v>
+        <v>-17.977932221868844</v>
       </c>
       <c r="H298">
-        <v>130.24318545304698</v>
+        <v>119.67814798329256</v>
       </c>
     </row>
     <row r="299" spans="2:8">
@@ -41563,19 +41563,19 @@
         <v>706</v>
       </c>
       <c r="C299">
-        <v>-12.690138373320879</v>
+        <v>-10.13254267953079</v>
       </c>
       <c r="D299">
-        <v>124.84028618906758</v>
+        <v>130.24318545304698</v>
       </c>
       <c r="F299" t="s">
         <v>1303</v>
       </c>
       <c r="G299">
-        <v>-12.690138373320879</v>
+        <v>-10.13254267953079</v>
       </c>
       <c r="H299">
-        <v>124.84028618906758</v>
+        <v>130.24318545304698</v>
       </c>
     </row>
     <row r="300" spans="2:8">
@@ -41583,19 +41583,19 @@
         <v>707</v>
       </c>
       <c r="C300">
-        <v>-43.459445564853546</v>
+        <v>-12.690138373320879</v>
       </c>
       <c r="D300">
-        <v>147.10370753016318</v>
+        <v>124.84028618906758</v>
       </c>
       <c r="F300" t="s">
         <v>1304</v>
       </c>
       <c r="G300">
-        <v>-43.459445564853546</v>
+        <v>-12.690138373320879</v>
       </c>
       <c r="H300">
-        <v>147.10370753016318</v>
+        <v>124.84028618906758</v>
       </c>
     </row>
     <row r="301" spans="2:8">

</xml_diff>

<commit_message>
Updated AUS_grids_kan50 model - 2026-09-09 09:14
</commit_message>
<xml_diff>
--- a/VerveStacks_AUS_grids_kan50/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_AUS_grids_kan50/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_AUS_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B9AE1DC-808B-463D-B7CF-FE7844B09502}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{000FA729-8C60-4454-9BF9-7DDA6EFAFE6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4932,7 +4932,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C9EB49D-E06F-478B-85C9-F18994D7B514}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F531D7D0-C54D-4ADE-83D9-4FAB56C671AE}">
   <dimension ref="B9:L302"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -35766,7 +35766,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2ADB422F-9FA9-4998-B303-561D311D6D69}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C42EF258-BCCC-4D2E-A4EF-BF6B6BB66303}">
   <dimension ref="B9:H302"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated AUS_grids_kan50 model - 2026-09-09 09:33
</commit_message>
<xml_diff>
--- a/VerveStacks_AUS_grids_kan50/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_AUS_grids_kan50/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_AUS_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{000FA729-8C60-4454-9BF9-7DDA6EFAFE6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9590F3A3-6379-46AB-B661-21DFB0F7AB94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4932,7 +4932,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F531D7D0-C54D-4ADE-83D9-4FAB56C671AE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFC7FA8B-1153-48C5-B5C9-DE05D6EA093B}">
   <dimension ref="B9:L302"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -35766,7 +35766,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C42EF258-BCCC-4D2E-A4EF-BF6B6BB66303}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3C6AF5A-9165-4D98-8DB5-A353763A3A50}">
   <dimension ref="B9:H302"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>